<commit_message>
Update invoice and transaction spreadsheets with latest data revisions
</commit_message>
<xml_diff>
--- a/data/invoices/totals.xlsx
+++ b/data/invoices/totals.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6160FED9-4F24-4E24-A06E-A2925FCC5166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFC2B88-9DE3-4E18-8A95-3659146753C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="الفواتير 2026-09-01 14-54" sheetId="1" r:id="rId1"/>
+    <sheet name="الفواتير 2026-09-07 10-53" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -208,7 +208,7 @@
     <t>2026-01-13</t>
   </si>
   <si>
-    <t>دنيا العوازال رقم الفاتورة 12.pdf</t>
+    <t>دنيا العوازل رقم الفاتورة 12.pdf</t>
   </si>
   <si>
     <t>12</t>
@@ -679,7 +679,7 @@
     <t>59753</t>
   </si>
   <si>
-    <t>دنيا العوازال رقم الفاتورة 60.pdf</t>
+    <t>دنيا العوازل رقم الفاتورة 60.pdf</t>
   </si>
   <si>
     <t>60</t>
@@ -1729,7 +1729,7 @@
     <t>FR003884-26</t>
   </si>
   <si>
-    <t>دنيا العوازال رقم الفاتورة 141.pdf</t>
+    <t>دنيا العوازل رقم الفاتورة 141.pdf</t>
   </si>
   <si>
     <t>2026-04-29</t>

</xml_diff>